<commit_message>
Restructure interface Include allocation acceptance/rejection message after Start Include Timer Change Pop up questions
</commit_message>
<xml_diff>
--- a/backend/tasks.xlsx
+++ b/backend/tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Zahra\PhD topic\Python\React\TaskMind\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mors/Develop/MasterThesis/Prototype/TaskMind/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91F7085-EDF9-448E-8F75-9327541E0540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A599CB-FBF2-FB4B-8806-2C2D4D11BFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -602,19 +602,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="3" width="53.5546875" customWidth="1"/>
-    <col min="4" max="5" width="28.21875" customWidth="1"/>
+    <col min="3" max="3" width="53.5" customWidth="1"/>
+    <col min="4" max="5" width="28.1640625" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" customWidth="1"/>
     <col min="7" max="7" width="11.6640625" customWidth="1"/>
-    <col min="8" max="8" width="28.109375" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" customWidth="1"/>
+    <col min="8" max="8" width="28.1640625" customWidth="1"/>
+    <col min="9" max="9" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -646,579 +646,561 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F2" s="4">
+        <v>52</v>
+      </c>
+      <c r="G2" s="4">
+        <v>32</v>
+      </c>
+      <c r="H2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="4">
-        <v>30</v>
-      </c>
-      <c r="H2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" s="2"/>
-      <c r="J2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <f>1+A2</f>
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>51</v>
-      </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F3" s="4">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="G3" s="4">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H3" t="s">
-        <v>51</v>
-      </c>
-      <c r="I3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <f t="shared" ref="A4:A20" si="0">1+A3</f>
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F4" s="4">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="G4" s="4">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
-      </c>
-      <c r="I4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="J4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
-        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>28</v>
+        <v>65</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
       </c>
       <c r="F5" s="4">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="G5" s="4">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H5" t="s">
         <v>39</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="J5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
-        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="4">
+        <v>35</v>
+      </c>
+      <c r="G6" s="4">
+        <v>30</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="4">
+        <v>20</v>
+      </c>
+      <c r="G7" s="4">
+        <v>100</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="21.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F8" s="1">
         <v>20</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G8" s="1">
         <v>30</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="J6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="4">
-        <v>10</v>
-      </c>
-      <c r="G7" s="4">
-        <v>30</v>
-      </c>
-      <c r="H7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="4">
-        <v>6</v>
-      </c>
-      <c r="G8" s="4">
-        <v>100</v>
-      </c>
-      <c r="H8" t="s">
-        <v>39</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="J8" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
-        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F9" s="4">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="J9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="4">
+        <v>6</v>
+      </c>
+      <c r="G10" s="4">
+        <v>100</v>
+      </c>
+      <c r="H10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="4">
+        <v>60</v>
+      </c>
+      <c r="G11" s="4">
+        <v>30</v>
+      </c>
+      <c r="H11" t="s">
+        <v>29</v>
+      </c>
+      <c r="J11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="4">
-        <v>12</v>
-      </c>
-      <c r="G10" s="4">
-        <v>25</v>
-      </c>
-      <c r="H10" t="s">
-        <v>41</v>
-      </c>
-      <c r="I10" t="s">
-        <v>12</v>
-      </c>
-      <c r="J10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="4">
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="4">
         <v>20</v>
       </c>
-      <c r="G11" s="4">
-        <v>32</v>
-      </c>
-      <c r="H11" t="s">
-        <v>15</v>
-      </c>
-      <c r="J11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F12" s="4">
-        <v>45</v>
-      </c>
       <c r="G12" s="4">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="H12" t="s">
         <v>39</v>
       </c>
       <c r="I12" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="J12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="E13" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="F13" s="4">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G13" s="4">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="H13" t="s">
         <v>39</v>
       </c>
       <c r="I13" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="J13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F14" s="4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G14" s="4">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="H14" t="s">
-        <v>39</v>
-      </c>
-      <c r="I14" t="s">
-        <v>36</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="I14" s="2"/>
       <c r="J14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F15" s="4">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="G15" s="4">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H15" t="s">
-        <v>21</v>
+        <v>51</v>
+      </c>
+      <c r="I15" t="s">
+        <v>23</v>
       </c>
       <c r="J15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E16" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F16" s="4">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="G16" s="4">
         <v>30</v>
       </c>
       <c r="H16" t="s">
-        <v>29</v>
+        <v>52</v>
+      </c>
+      <c r="I16" t="s">
+        <v>23</v>
       </c>
       <c r="J16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="F17" s="4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G17" s="4">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="H17" t="s">
         <v>39</v>
       </c>
       <c r="I17" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="J17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="F18" s="4">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="G18" s="4">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="H18" t="s">
-        <v>39</v>
-      </c>
-      <c r="I18" t="s">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="J18" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="F19" s="4">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="G19" s="4">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H19" t="s">
-        <v>6</v>
+        <v>41</v>
+      </c>
+      <c r="I19" t="s">
+        <v>12</v>
       </c>
       <c r="J19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B20" t="s">
@@ -1246,28 +1228,26 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1E446E5-85DE-4FD9-98F7-92D9EA47C386}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="20.109375" customWidth="1"/>
-    <col min="3" max="3" width="27.88671875" customWidth="1"/>
-    <col min="4" max="4" width="21.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" customWidth="1"/>
+    <col min="3" max="3" width="27.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.5" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" customWidth="1"/>
-    <col min="7" max="7" width="28.77734375" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
     <col min="8" max="8" width="52.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1299,7 +1279,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1329,7 +1309,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <f>1+A2</f>
         <v>2</v>
@@ -1362,7 +1342,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <f t="shared" ref="A4:A6" si="0">1+A3</f>
         <v>3</v>
@@ -1395,7 +1375,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1428,7 +1408,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <f t="shared" si="0"/>
         <v>5</v>

</xml_diff>